<commit_message>
fix(backend): fix phone regex, date calculation & update BVA/EP point
</commit_message>
<xml_diff>
--- a/docs/testing/BVA/Auth/Auth_User_BVA_TestCases_4n1.xlsx
+++ b/docs/testing/BVA/Auth/Auth_User_BVA_TestCases_4n1.xlsx
@@ -581,7 +581,7 @@
           <t>{
   "fullName": "Nguyen Van Nominal",
   "email": "nominal_{{dyn_ts}}@gmail.com",
-  "phone": "090{{dyn_ts}}",
+  "phone": "09{{dyn_ts}}",
   "username": "nom_{{dyn_ts}}",
   "password": "PassNominal123"
 }</t>
@@ -645,7 +645,7 @@
           <t>{
   "fullName": "A",
   "email": "fn1_{{dyn_ts}}@gmail.com",
-  "phone": "091{{dyn_ts}}",
+  "phone": "09{{dyn_ts}}",
   "username": "u1_{{dyn_ts}}",
   "password": "PassNominal123"
 }</t>
@@ -709,7 +709,7 @@
           <t>{
   "fullName": "An",
   "email": "fn2_{{dyn_ts}}@gmail.com",
-  "phone": "092{{dyn_ts}}",
+  "phone": "09{{dyn_ts}}",
   "username": "u2_{{dyn_ts}}",
   "password": "PassNominal123"
 }</t>
@@ -773,7 +773,7 @@
           <t>{
   "fullName": "{{fn_99}}",
   "email": "fn99_{{dyn_ts}}@gmail.com",
-  "phone": "093{{dyn_ts}}",
+  "phone": "09{{dyn_ts}}",
   "username": "u99_{{dyn_ts}}",
   "password": "PassNominal123"
 }</t>
@@ -837,7 +837,7 @@
           <t>{
   "fullName": "{{fn_100}}",
   "email": "fn100_{{dyn_ts}}@gmail.com",
-  "phone": "094{{dyn_ts}}",
+  "phone": "09{{dyn_ts}}",
   "username": "u100_{{dyn_ts}}",
   "password": "PassNominal123"
 }</t>
@@ -901,7 +901,7 @@
           <t>{
   "fullName": "Nguyen Van Nominal",
   "email": "un1_{{dyn_ts}}@gmail.com",
-  "phone": "095{{dyn_ts}}",
+  "phone": "09{{dyn_ts}}",
   "username": "{{un_1}}",
   "password": "PassNominal123"
 }</t>
@@ -965,7 +965,7 @@
           <t>{
   "fullName": "Nguyen Van Nominal",
   "email": "un2_{{dyn_ts}}@gmail.com",
-  "phone": "096{{dyn_ts}}",
+  "phone": "09{{dyn_ts}}",
   "username": "{{un_2}}",
   "password": "PassNominal123"
 }</t>
@@ -1029,7 +1029,7 @@
           <t>{
   "fullName": "Nguyen Van Nominal",
   "email": "un39_{{dyn_ts}}@gmail.com",
-  "phone": "097{{dyn_ts}}",
+  "phone": "09{{dyn_ts}}",
   "username": "{{un_39}}",
   "password": "PassNominal123"
 }</t>
@@ -1093,7 +1093,7 @@
           <t>{
   "fullName": "Nguyen Van Nominal",
   "email": "un40_{{dyn_ts}}@gmail.com",
-  "phone": "098{{dyn_ts}}",
+  "phone": "09{{dyn_ts}}",
   "username": "{{un_40}}",
   "password": "PassNominal123"
 }</t>
@@ -1137,7 +1137,7 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>password Biên dưới: Min = 6 ký tự ('123456')</t>
+          <t>password Biên dưới: Min = 8 ký tự ('Pass1234')</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
@@ -1148,7 +1148,7 @@
       <c r="D11" s="6" t="inlineStr">
         <is>
           <t>1. POST /api/auth/register
-2. Gửi password=6 chars
+2. Gửi password=8 chars
 3. Kiểm tra status 201</t>
         </is>
       </c>
@@ -1156,17 +1156,17 @@
         <is>
           <t>{
   "fullName": "Nguyen Van Nominal",
-  "email": "p6_{{dyn_ts}}@gmail.com",
-  "phone": "081{{dyn_ts}}",
-  "username": "p6_{{dyn_ts}}",
-  "password": "123456"
+  "email": "p8_{{dyn_ts}}@gmail.com",
+  "phone": "09{{dyn_ts}}",
+  "username": "p8_{{dyn_ts}}",
+  "password": "Pass1234"
 }</t>
         </is>
       </c>
       <c r="F11" s="6" t="inlineStr">
         <is>
           <t>Status: 201 Created
-Đăng ký thành công với password 6 ký tự.</t>
+Đăng ký thành công với password 8 ký tự.</t>
         </is>
       </c>
       <c r="G11" s="6" t="inlineStr">
@@ -1201,7 +1201,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>password Biên dưới + 1: Min+1 = 7 ký tự ('1234567')</t>
+          <t>password Biên dưới + 1: Min+1 = 9 ký tự ('Pass12345')</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -1212,7 +1212,7 @@
       <c r="D12" s="3" t="inlineStr">
         <is>
           <t>1. POST /api/auth/register
-2. Gửi password=7 chars
+2. Gửi password=9 chars
 3. Kiểm tra status 201</t>
         </is>
       </c>
@@ -1220,17 +1220,17 @@
         <is>
           <t>{
   "fullName": "Nguyen Van Nominal",
-  "email": "p7_{{dyn_ts}}@gmail.com",
-  "phone": "082{{dyn_ts}}",
-  "username": "p7_{{dyn_ts}}",
-  "password": "1234567"
+  "email": "p9_{{dyn_ts}}@gmail.com",
+  "phone": "09{{dyn_ts}}",
+  "username": "p9_{{dyn_ts}}",
+  "password": "Pass12345"
 }</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
           <t>Status: 201 Created
-Đăng ký thành công với password 7 ký tự.</t>
+Đăng ký thành công với password 9 ký tự.</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
@@ -1265,7 +1265,7 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>password Biên trên - 1: Max-1 = 15 ký tự</t>
+          <t>password Biên trên - 1: Max-1 = 15 ký tự ('Pass15chars_123')</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
@@ -1285,7 +1285,7 @@
           <t>{
   "fullName": "Nguyen Van Nominal",
   "email": "p15_{{dyn_ts}}@gmail.com",
-  "phone": "083{{dyn_ts}}",
+  "phone": "09{{dyn_ts}}",
   "username": "p15_{{dyn_ts}}",
   "password": "Pass15chars_123"
 }</t>
@@ -1329,7 +1329,7 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>password Biên trên: Max = 16 ký tự</t>
+          <t>password Biên trên: Max = 16 ký tự ('Pass16chars_1234')</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
@@ -1349,7 +1349,7 @@
           <t>{
   "fullName": "Nguyen Van Nominal",
   "email": "p16_{{dyn_ts}}@gmail.com",
-  "phone": "084{{dyn_ts}}",
+  "phone": "09{{dyn_ts}}",
   "username": "p16_{{dyn_ts}}",
   "password": "Pass16chars_1234"
 }</t>
@@ -1393,7 +1393,7 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>phone Biên dưới: Min = 9 số ('091234567')</t>
+          <t>phone Biên dưới: Min = 10 số ('0912345678')</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
@@ -1402,77 +1402,13 @@
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
-        <is>
-          <t>1. POST /api/auth/register
-2. Gửi phone=9 digits
-3. Kiểm tra status 201</t>
-        </is>
-      </c>
-      <c r="E15" s="6" t="inlineStr">
-        <is>
-          <t>{
-  "fullName": "Nguyen Van Nominal",
-  "email": "ph9_{{dyn_ts}}@gmail.com",
-  "phone": "{{ph_9}}",
-  "username": "ph9_{{dyn_ts}}",
-  "password": "PassNominal123"
-}</t>
-        </is>
-      </c>
-      <c r="F15" s="6" t="inlineStr">
-        <is>
-          <t>Status: 201 Created
-Đăng ký thành công với số điện thoại 9 số.</t>
-        </is>
-      </c>
-      <c r="G15" s="6" t="inlineStr">
-        <is>
-          <t>HTTP 201 Created. Đăng ký thành công.</t>
-        </is>
-      </c>
-      <c r="H15" s="4" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="I15" s="5" t="n">
-        <v>80</v>
-      </c>
-      <c r="J15" s="5" t="inlineStr">
-        <is>
-          <t>POST</t>
-        </is>
-      </c>
-      <c r="K15" s="6" t="inlineStr">
-        <is>
-          <t>/api/auth/register</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>TC_BVA_REG_014</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>phone Biên dưới + 1: Min+1 = 10 số ('0912345678')</t>
-        </is>
-      </c>
-      <c r="C16" s="3" t="inlineStr">
-        <is>
-          <t>Server Backend đang chạy.</t>
-        </is>
-      </c>
-      <c r="D16" s="3" t="inlineStr">
         <is>
           <t>1. POST /api/auth/register
 2. Gửi phone=10 digits
 3. Kiểm tra status 201</t>
         </is>
       </c>
-      <c r="E16" s="3" t="inlineStr">
+      <c r="E15" s="6" t="inlineStr">
         <is>
           <t>{
   "fullName": "Nguyen Van Nominal",
@@ -1483,60 +1419,60 @@
 }</t>
         </is>
       </c>
-      <c r="F16" s="3" t="inlineStr">
+      <c r="F15" s="6" t="inlineStr">
         <is>
           <t>Status: 201 Created
 Đăng ký thành công với số điện thoại 10 số.</t>
         </is>
       </c>
-      <c r="G16" s="3" t="inlineStr">
+      <c r="G15" s="6" t="inlineStr">
         <is>
           <t>HTTP 201 Created. Đăng ký thành công.</t>
         </is>
       </c>
-      <c r="H16" s="4" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="I16" s="2" t="n">
-        <v>82</v>
-      </c>
-      <c r="J16" s="2" t="inlineStr">
-        <is>
-          <t>POST</t>
-        </is>
-      </c>
-      <c r="K16" s="3" t="inlineStr">
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I15" s="5" t="n">
+        <v>80</v>
+      </c>
+      <c r="J15" s="5" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="K15" s="6" t="inlineStr">
         <is>
           <t>/api/auth/register</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t>TC_BVA_REG_015</t>
-        </is>
-      </c>
-      <c r="B17" s="6" t="inlineStr">
-        <is>
-          <t>phone Biên trên - 1: Max-1 = 11 số ('09123456789')</t>
-        </is>
-      </c>
-      <c r="C17" s="6" t="inlineStr">
-        <is>
-          <t>Server Backend đang chạy.</t>
-        </is>
-      </c>
-      <c r="D17" s="6" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>TC_BVA_REG_014</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>phone Biên dưới + 1: Min+1 = 11 số ('09123456789')</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Server Backend đang chạy.</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
         <is>
           <t>1. POST /api/auth/register
 2. Gửi phone=11 digits
 3. Kiểm tra status 201</t>
         </is>
       </c>
-      <c r="E17" s="6" t="inlineStr">
+      <c r="E16" s="3" t="inlineStr">
         <is>
           <t>{
   "fullName": "Nguyen Van Nominal",
@@ -1547,6 +1483,70 @@
 }</t>
         </is>
       </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>Status: 201 Created
+Đăng ký thành công với số điện thoại 11 số.</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>HTTP 201 Created. Đăng ký thành công.</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="n">
+        <v>82</v>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="K16" s="3" t="inlineStr">
+        <is>
+          <t>/api/auth/register</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>TC_BVA_REG_015</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>phone Biên trên - 1: Max-1 = 11 số ('09123456789')</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>Server Backend đang chạy.</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>1. POST /api/auth/register
+2. Gửi phone=11 digits
+3. Kiểm tra status 201</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>{
+  "fullName": "Nguyen Van Nominal",
+  "email": "ph11_{{dyn_ts}}@gmail.com",
+  "phone": "{{ph_11}}",
+  "username": "ph11_{{dyn_ts}}",
+  "password": "PassNominal123"
+}</t>
+        </is>
+      </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
           <t>Status: 201 Created
@@ -1669,7 +1669,7 @@
           <t>{
   "fullName": "Nguyen Van Nominal",
   "email": "{{em_10}}",
-  "phone": "085{{dyn_ts}}",
+  "phone": "09{{dyn_ts}}",
   "username": "em10_{{dyn_ts}}",
   "password": "PassNominal123"
 }</t>
@@ -1733,7 +1733,7 @@
           <t>{
   "fullName": "Nguyen Van Nominal",
   "email": "{{em_11}}",
-  "phone": "086{{dyn_ts}}",
+  "phone": "09{{dyn_ts}}",
   "username": "em11_{{dyn_ts}}",
   "password": "PassNominal123"
 }</t>
@@ -1797,7 +1797,7 @@
           <t>{
   "fullName": "Nguyen Van Nominal",
   "email": "{{em_99}}",
-  "phone": "087{{dyn_ts}}",
+  "phone": "09{{dyn_ts}}",
   "username": "em99_{{dyn_ts}}",
   "password": "PassNominal123"
 }</t>
@@ -1861,7 +1861,7 @@
           <t>{
   "fullName": "Nguyen Van Nominal",
   "email": "{{em_100}}",
-  "phone": "088{{dyn_ts}}",
+  "phone": "09{{dyn_ts}}",
   "username": "em100_{{dyn_ts}}",
   "password": "PassNominal123"
 }</t>
@@ -2210,7 +2210,7 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>password Biên dưới: Min = 6 ký tự ('123456')</t>
+          <t>password Biên dưới: Min = 8 ký tự ('Pass1234')</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
@@ -2221,7 +2221,7 @@
       <c r="D28" s="3" t="inlineStr">
         <is>
           <t>1. POST /api/auth/login
-2. Gửi password=6 chars
+2. Gửi password=8 chars
 3. Kiểm tra phản hồi</t>
         </is>
       </c>
@@ -2229,7 +2229,7 @@
         <is>
           <t>{
   "account": "admin",
-  "password": "123456"
+  "password": "Pass1234"
 }</t>
         </is>
       </c>
@@ -2271,7 +2271,7 @@
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>password Biên dưới + 1: Min+1 = 7 ký tự ('1234567')</t>
+          <t>password Biên dưới + 1: Min+1 = 9 ký tự ('Pass12345')</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
@@ -2282,7 +2282,7 @@
       <c r="D29" s="6" t="inlineStr">
         <is>
           <t>1. POST /api/auth/login
-2. Gửi password=7 chars
+2. Gửi password=9 chars
 3. Kiểm tra phản hồi</t>
         </is>
       </c>
@@ -2290,7 +2290,7 @@
         <is>
           <t>{
   "account": "admin",
-  "password": "1234567"
+  "password": "Pass12345"
 }</t>
         </is>
       </c>
@@ -2332,7 +2332,7 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>password Biên trên - 1: Max-1 = 15 ký tự</t>
+          <t>password Biên trên - 1: Max-1 = 15 ký tự ('Pass15chars_123')</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
@@ -2393,7 +2393,7 @@
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>password Biên trên: Max = 16 ký tự</t>
+          <t>password Biên trên: Max = 16 ký tự ('Pass16chars_1234')</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">

</xml_diff>